<commit_message>
■MET-S_ADBZR-CSTD対応 BEV3CDCMET-3682 BEV3CDCMET-1009 【コンポーネント】 Alert パラメータ設定書のReferenceシート修正
</commit_message>
<xml_diff>
--- a/src/PE1VM1/App/MET/IpcApplication/Vom/Alert/matrix/scc/alert_S_ADBZR_ACC-CSTD-0-06-A-C0.xlsx
+++ b/src/PE1VM1/App/MET/IpcApplication/Vom/Alert/matrix/scc/alert_S_ADBZR_ACC-CSTD-0-06-A-C0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.91.244.104\body-ph\DTPH資産(製品別)\グラフィック\業務管理\SINGLETASK_FY25\32_BEV_MCU_シス検ADAS向け_設計サポート\03_Output\07_Alertマクロ変更(ADBZR)\crosschecked_assasin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\s10035azcfs0534.file.core.windows.net\metersoft\開発用\Toyota\BEV\設計成果物_MET\MCU-DT\02.Design\06.FF2\A1.要件\BEV3CDCMET-3653_S_ADBZR\01.パラメータ設計書\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E96A0646-C209-4ED7-91A1-32F7CE59A432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11445158-1E2F-4154-858A-75BAC90A5847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-2250" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="表紙（承認欄）" sheetId="17" r:id="rId1"/>
@@ -5961,37 +5961,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="19" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="19" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6036,10 +6015,31 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -6305,14 +6305,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>34</xdr:col>
       <xdr:colOff>46727</xdr:colOff>
       <xdr:row>51</xdr:row>
       <xdr:rowOff>7397</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>94576</xdr:colOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>94575</xdr:colOff>
       <xdr:row>53</xdr:row>
       <xdr:rowOff>170667</xdr:rowOff>
     </xdr:to>
@@ -6344,8 +6344,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5223845" y="8938485"/>
-          <a:ext cx="518496" cy="561415"/>
+          <a:off x="5761727" y="9117779"/>
+          <a:ext cx="552113" cy="566682"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6519,15 +6519,15 @@
       <xdr:twoCellAnchor editAs="absolute">
         <xdr:from>
           <xdr:col>35</xdr:col>
-          <xdr:colOff>67010</xdr:colOff>
+          <xdr:colOff>167528</xdr:colOff>
           <xdr:row>53</xdr:row>
-          <xdr:rowOff>51997</xdr:rowOff>
+          <xdr:rowOff>79561</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>38</xdr:col>
-          <xdr:colOff>111679</xdr:colOff>
+          <xdr:col>39</xdr:col>
+          <xdr:colOff>47065</xdr:colOff>
           <xdr:row>55</xdr:row>
-          <xdr:rowOff>177390</xdr:rowOff>
+          <xdr:rowOff>193861</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -6537,7 +6537,7 @@
                   <a14:compatExt spid="_x0000_s1025"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4C2DCB5-8F03-791C-7894-E9D80A7EE978}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -6555,7 +6555,6 @@
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
             <a:extLst>
               <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
                 <a14:hiddenFill>
@@ -6569,20 +6568,10 @@
                   <a:solidFill>
                     <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
                   </a:solidFill>
-                  <a:prstDash val="solid"/>
                   <a:miter lim="800000"/>
                   <a:headEnd/>
-                  <a:tailEnd type="none" w="med" len="med"/>
+                  <a:tailEnd/>
                 </a14:hiddenLine>
-              </a:ext>
-              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-                <a14:hiddenEffects>
-                  <a:effectLst>
-                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="808080"/>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </a14:hiddenEffects>
               </a:ext>
             </a:extLst>
           </xdr:spPr>
@@ -7956,7 +7945,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>35</xdr:col>
-      <xdr:colOff>522867</xdr:colOff>
+      <xdr:colOff>593912</xdr:colOff>
       <xdr:row>98</xdr:row>
       <xdr:rowOff>112059</xdr:rowOff>
     </xdr:to>
@@ -7973,8 +7962,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="40620353" y="8602638"/>
-          <a:ext cx="1072926" cy="11220568"/>
+          <a:off x="45394059" y="8602638"/>
+          <a:ext cx="1222412" cy="11299009"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8016,13 +8005,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>38</xdr:col>
-      <xdr:colOff>571744</xdr:colOff>
+      <xdr:colOff>605119</xdr:colOff>
       <xdr:row>100</xdr:row>
       <xdr:rowOff>63558</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>43</xdr:col>
-      <xdr:colOff>394111</xdr:colOff>
+      <xdr:colOff>392207</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>44823</xdr:rowOff>
     </xdr:to>
@@ -8039,8 +8028,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="43557509" y="20110882"/>
-          <a:ext cx="2847955" cy="821706"/>
+          <a:off x="48678354" y="20189323"/>
+          <a:ext cx="3204882" cy="821706"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8724,72 +8713,6 @@
             <a:latin typeface="Meiryo UI" panose="020B0604030504040204" pitchFamily="50" charset="-128"/>
             <a:ea typeface="Meiryo UI" panose="020B0604030504040204" pitchFamily="50" charset="-128"/>
           </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>95699</xdr:colOff>
-      <xdr:row>114</xdr:row>
-      <xdr:rowOff>114944</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>151216</xdr:colOff>
-      <xdr:row>115</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="166" name="正方形/長方形 165">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0B00-0000A6000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="41919108" y="22974944"/>
-          <a:ext cx="661653" cy="132360"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="38100">
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -9663,19 +9586,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DFC1F9F-09B5-4CC2-988E-73D785546469}">
   <dimension ref="T13:AM56"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="39" width="2.21875" style="228" customWidth="1"/>
+    <col min="1" max="39" width="2.25" style="228" customWidth="1"/>
     <col min="40" max="16384" width="9" style="228"/>
   </cols>
   <sheetData>
     <row r="13" spans="20:20">
       <c r="T13" s="227" t="str">
         <f ca="1">LEFT(MID(CELL("filename"),FIND("[",CELL("filename"))+1,FIND("]",CELL("filename"))-FIND("[",CELL("filename"))-1),LEN(MID(CELL("filename"),FIND("[",CELL("filename"))+1,FIND("]",CELL("filename"))-FIND("[",CELL("filename"))-1))-5)</f>
-        <v>BEV_シス検ADAS_BEV3CDCMET-2019_ICEテスト</v>
-      </c>
-    </row>
-    <row r="34" spans="25:39" ht="15">
+        <v>alert_S_ADBZR_ACC-CSTD-0-06-A-C0</v>
+      </c>
+    </row>
+    <row r="34" spans="25:39" ht="15.75">
       <c r="Y34" s="260" t="s">
         <v>319</v>
       </c>
@@ -9694,7 +9617,7 @@
       <c r="AL34" s="244"/>
       <c r="AM34" s="244"/>
     </row>
-    <row r="35" spans="25:39" ht="15">
+    <row r="35" spans="25:39" ht="15.75">
       <c r="Y35" s="283" t="s">
         <v>300</v>
       </c>
@@ -9717,7 +9640,7 @@
       <c r="AL35" s="284"/>
       <c r="AM35" s="285"/>
     </row>
-    <row r="36" spans="25:39" ht="15">
+    <row r="36" spans="25:39" ht="15.75">
       <c r="Y36" s="245"/>
       <c r="Z36" s="246"/>
       <c r="AA36" s="246"/>
@@ -9734,7 +9657,7 @@
       <c r="AL36" s="246"/>
       <c r="AM36" s="247"/>
     </row>
-    <row r="37" spans="25:39" ht="15">
+    <row r="37" spans="25:39" ht="15.75">
       <c r="Y37" s="248"/>
       <c r="Z37" s="244"/>
       <c r="AA37" s="244"/>
@@ -9751,7 +9674,7 @@
       <c r="AL37" s="244"/>
       <c r="AM37" s="249"/>
     </row>
-    <row r="38" spans="25:39" ht="15">
+    <row r="38" spans="25:39" ht="15.75">
       <c r="Y38" s="248"/>
       <c r="Z38" s="250"/>
       <c r="AA38" s="251" t="s">
@@ -9774,7 +9697,7 @@
       <c r="AL38" s="250"/>
       <c r="AM38" s="252"/>
     </row>
-    <row r="39" spans="25:39" ht="15">
+    <row r="39" spans="25:39" ht="15.75">
       <c r="Y39" s="248"/>
       <c r="Z39" s="244"/>
       <c r="AA39" s="244"/>
@@ -9791,7 +9714,7 @@
       <c r="AL39" s="244"/>
       <c r="AM39" s="249"/>
     </row>
-    <row r="40" spans="25:39" ht="15">
+    <row r="40" spans="25:39" ht="15.75">
       <c r="Y40" s="254"/>
       <c r="Z40" s="255"/>
       <c r="AA40" s="255"/>
@@ -9808,7 +9731,7 @@
       <c r="AL40" s="255"/>
       <c r="AM40" s="256"/>
     </row>
-    <row r="41" spans="25:39" ht="15">
+    <row r="41" spans="25:39" ht="15.75">
       <c r="Y41" s="244"/>
       <c r="Z41" s="244"/>
       <c r="AA41" s="244"/>
@@ -9825,7 +9748,7 @@
       <c r="AL41" s="244"/>
       <c r="AM41" s="244"/>
     </row>
-    <row r="42" spans="25:39" ht="15">
+    <row r="42" spans="25:39" ht="15.75">
       <c r="Y42" s="260" t="s">
         <v>320</v>
       </c>
@@ -9844,7 +9767,7 @@
       <c r="AL42" s="244"/>
       <c r="AM42" s="244"/>
     </row>
-    <row r="43" spans="25:39" ht="15">
+    <row r="43" spans="25:39" ht="15.75">
       <c r="Y43" s="283" t="s">
         <v>300</v>
       </c>
@@ -9867,7 +9790,7 @@
       <c r="AL43" s="284"/>
       <c r="AM43" s="285"/>
     </row>
-    <row r="44" spans="25:39" ht="15">
+    <row r="44" spans="25:39" ht="15.75">
       <c r="Y44" s="245"/>
       <c r="Z44" s="246"/>
       <c r="AA44" s="246"/>
@@ -9884,7 +9807,7 @@
       <c r="AL44" s="246"/>
       <c r="AM44" s="247"/>
     </row>
-    <row r="45" spans="25:39" ht="15">
+    <row r="45" spans="25:39" ht="15.75">
       <c r="Y45" s="248"/>
       <c r="Z45" s="244"/>
       <c r="AA45" s="244"/>
@@ -9901,7 +9824,7 @@
       <c r="AL45" s="244"/>
       <c r="AM45" s="249"/>
     </row>
-    <row r="46" spans="25:39" ht="15">
+    <row r="46" spans="25:39" ht="15.75">
       <c r="Y46" s="248"/>
       <c r="Z46" s="250"/>
       <c r="AA46" s="251" t="s">
@@ -9924,7 +9847,7 @@
       <c r="AL46" s="250"/>
       <c r="AM46" s="252"/>
     </row>
-    <row r="47" spans="25:39" ht="15">
+    <row r="47" spans="25:39" ht="15.75">
       <c r="Y47" s="248"/>
       <c r="Z47" s="244"/>
       <c r="AA47" s="244"/>
@@ -9941,7 +9864,7 @@
       <c r="AL47" s="244"/>
       <c r="AM47" s="249"/>
     </row>
-    <row r="48" spans="25:39" ht="15">
+    <row r="48" spans="25:39" ht="15.75">
       <c r="Y48" s="254"/>
       <c r="Z48" s="255"/>
       <c r="AA48" s="255"/>
@@ -9958,7 +9881,7 @@
       <c r="AL48" s="255"/>
       <c r="AM48" s="256"/>
     </row>
-    <row r="50" spans="25:39" ht="15">
+    <row r="50" spans="25:39" ht="15.75">
       <c r="Y50" s="243" t="s">
         <v>314</v>
       </c>
@@ -9986,7 +9909,7 @@
       <c r="AL51" s="281"/>
       <c r="AM51" s="282"/>
     </row>
-    <row r="52" spans="25:39" ht="15">
+    <row r="52" spans="25:39" ht="15.75">
       <c r="Y52" s="245"/>
       <c r="Z52" s="246"/>
       <c r="AA52" s="246"/>
@@ -10003,7 +9926,7 @@
       <c r="AL52" s="231"/>
       <c r="AM52" s="232"/>
     </row>
-    <row r="53" spans="25:39" ht="15">
+    <row r="53" spans="25:39" ht="15.75">
       <c r="Y53" s="248"/>
       <c r="Z53" s="244"/>
       <c r="AA53" s="244"/>
@@ -10018,7 +9941,7 @@
       <c r="AK53" s="229"/>
       <c r="AM53" s="234"/>
     </row>
-    <row r="54" spans="25:39" ht="15">
+    <row r="54" spans="25:39" ht="15.75">
       <c r="Y54" s="253"/>
       <c r="Z54" s="250"/>
       <c r="AA54" s="251" t="s">
@@ -10039,7 +9962,7 @@
       <c r="AL54" s="235"/>
       <c r="AM54" s="237"/>
     </row>
-    <row r="55" spans="25:39" ht="15">
+    <row r="55" spans="25:39" ht="15.75">
       <c r="Y55" s="248"/>
       <c r="Z55" s="244"/>
       <c r="AA55" s="244"/>
@@ -10053,7 +9976,7 @@
       <c r="AI55" s="233"/>
       <c r="AM55" s="234"/>
     </row>
-    <row r="56" spans="25:39" ht="15">
+    <row r="56" spans="25:39" ht="15.75">
       <c r="Y56" s="254"/>
       <c r="Z56" s="255"/>
       <c r="AA56" s="255"/>
@@ -10095,15 +10018,15 @@
             <anchor>
               <from>
                 <xdr:col>35</xdr:col>
-                <xdr:colOff>68580</xdr:colOff>
+                <xdr:colOff>171450</xdr:colOff>
                 <xdr:row>53</xdr:row>
-                <xdr:rowOff>53340</xdr:rowOff>
+                <xdr:rowOff>76200</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>38</xdr:col>
-                <xdr:colOff>114300</xdr:colOff>
+                <xdr:col>39</xdr:col>
+                <xdr:colOff>47625</xdr:colOff>
                 <xdr:row>55</xdr:row>
-                <xdr:rowOff>175260</xdr:rowOff>
+                <xdr:rowOff>190500</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -10121,15 +10044,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:X19"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="4.44140625" customWidth="1"/>
+    <col min="1" max="1" width="4.5" customWidth="1"/>
     <col min="2" max="2" width="9" style="9" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="72.88671875" customWidth="1"/>
-    <col min="5" max="6" width="12.77734375" customWidth="1"/>
-    <col min="7" max="18" width="13.109375" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="72.875" customWidth="1"/>
+    <col min="5" max="6" width="12.75" customWidth="1"/>
+    <col min="7" max="18" width="13.125" hidden="1" customWidth="1"/>
     <col min="19" max="22" width="0" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:24" ht="25.5" customHeight="1">
@@ -10199,7 +10122,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:24" ht="13.8" thickBot="1"/>
+    <row r="6" spans="2:24" ht="14.25" thickBot="1"/>
     <row r="7" spans="2:24">
       <c r="C7" s="292" t="s">
         <v>0</v>
@@ -10234,7 +10157,7 @@
       <c r="W7" s="290"/>
       <c r="X7" s="291"/>
     </row>
-    <row r="8" spans="2:24" ht="27" thickBot="1">
+    <row r="8" spans="2:24" ht="27.75" thickBot="1">
       <c r="B8" s="9" t="s">
         <v>91</v>
       </c>
@@ -10305,7 +10228,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:24" ht="209.4" customHeight="1" thickTop="1">
+    <row r="9" spans="2:24" ht="209.45" customHeight="1" thickTop="1">
       <c r="B9" s="9">
         <f t="shared" ref="B9:B15" si="0">IF(C9=0,0,ROW()-ROW($B$8))</f>
         <v>1</v>
@@ -10361,7 +10284,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:24" ht="212.4" customHeight="1">
+    <row r="10" spans="2:24" ht="212.45" customHeight="1">
       <c r="B10" s="9">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -10417,7 +10340,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="2:24" ht="145.19999999999999" customHeight="1">
+    <row r="11" spans="2:24" ht="145.15" customHeight="1">
       <c r="B11" s="9">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10753,7 +10676,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="2:24" ht="26.4">
+    <row r="17" spans="2:24" ht="27">
       <c r="B17" s="9">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -10789,7 +10712,7 @@
         <v>45387</v>
       </c>
     </row>
-    <row r="18" spans="2:24" ht="264">
+    <row r="18" spans="2:24" ht="270">
       <c r="B18" s="9">
         <f t="shared" ref="B18" si="3">IF(C18=0,0,ROW()-ROW($B$8))</f>
         <v>10</v>
@@ -10845,7 +10768,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="2:24" ht="145.19999999999999">
+    <row r="19" spans="2:24" ht="148.5">
       <c r="C19" s="261" t="s">
         <v>338</v>
       </c>
@@ -10917,11 +10840,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="B2:E39"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="4.6640625" customWidth="1"/>
-    <col min="3" max="3" width="3.44140625" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="4.625" customWidth="1"/>
+    <col min="3" max="3" width="3.5" customWidth="1"/>
+    <col min="4" max="4" width="17.5" customWidth="1"/>
     <col min="5" max="5" width="106" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10935,13 +10858,13 @@
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="13.8" thickBot="1">
+    <row r="6" spans="2:5" ht="14.25" thickBot="1">
       <c r="B6" s="138" t="s">
         <v>129</v>
       </c>
       <c r="C6" s="138"/>
     </row>
-    <row r="7" spans="2:5" ht="13.8" thickBot="1">
+    <row r="7" spans="2:5" ht="14.25" thickBot="1">
       <c r="C7" s="68" t="s">
         <v>131</v>
       </c>
@@ -10966,7 +10889,7 @@
       <c r="D9" s="149"/>
       <c r="E9" s="148"/>
     </row>
-    <row r="10" spans="2:5" ht="13.8" thickBot="1">
+    <row r="10" spans="2:5" ht="14.25" thickBot="1">
       <c r="C10" s="145"/>
       <c r="D10" s="79"/>
       <c r="E10" s="5"/>
@@ -10974,14 +10897,14 @@
     <row r="11" spans="2:5">
       <c r="C11" s="143"/>
     </row>
-    <row r="12" spans="2:5" ht="13.8" thickBot="1">
+    <row r="12" spans="2:5" ht="14.25" thickBot="1">
       <c r="B12" s="139" t="s">
         <v>130</v>
       </c>
       <c r="C12" s="75"/>
       <c r="D12" s="75"/>
     </row>
-    <row r="13" spans="2:5" ht="13.8" thickBot="1">
+    <row r="13" spans="2:5" ht="14.25" thickBot="1">
       <c r="B13" s="140"/>
       <c r="C13" s="144" t="s">
         <v>131</v>
@@ -10993,7 +10916,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="13.8" thickTop="1">
+    <row r="14" spans="2:5" ht="14.25" thickTop="1">
       <c r="C14" s="141">
         <v>0</v>
       </c>
@@ -11070,17 +10993,17 @@
         <v>163</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="13.8" thickBot="1">
+    <row r="21" spans="2:5" ht="14.25" thickBot="1">
       <c r="C21" s="145"/>
       <c r="D21" s="79"/>
       <c r="E21" s="5"/>
     </row>
-    <row r="24" spans="2:5" ht="13.8" thickBot="1">
+    <row r="24" spans="2:5" ht="14.25" thickBot="1">
       <c r="B24" s="138" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="2:5" ht="13.8" thickBot="1">
+    <row r="25" spans="2:5" ht="14.25" thickBot="1">
       <c r="C25" s="144" t="s">
         <v>131</v>
       </c>
@@ -11167,12 +11090,12 @@
       <c r="D33" s="78"/>
       <c r="E33" s="67"/>
     </row>
-    <row r="34" spans="2:5" ht="13.8" thickBot="1">
+    <row r="34" spans="2:5" ht="14.25" thickBot="1">
       <c r="C34" s="145"/>
       <c r="D34" s="79"/>
       <c r="E34" s="5"/>
     </row>
-    <row r="37" spans="2:5" ht="13.8" thickBot="1">
+    <row r="37" spans="2:5" ht="14.25" thickBot="1">
       <c r="B37" s="138" t="s">
         <v>159</v>
       </c>
@@ -11184,7 +11107,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="2:5" ht="13.8" thickBot="1">
+    <row r="39" spans="2:5" ht="14.25" thickBot="1">
       <c r="C39" s="300"/>
       <c r="D39" s="301"/>
       <c r="E39" s="5" t="s">
@@ -11211,132 +11134,132 @@
     <tabColor rgb="FFCCFFCC"/>
   </sheetPr>
   <dimension ref="B1:O37"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="3.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="26.77734375" customWidth="1"/>
-    <col min="9" max="9" width="20.88671875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="3.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="26.75" customWidth="1"/>
+    <col min="9" max="9" width="20.875" hidden="1" customWidth="1"/>
     <col min="10" max="14" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" ht="13.8" thickBot="1"/>
+    <row r="1" spans="2:15" ht="14.25" thickBot="1"/>
     <row r="2" spans="2:15">
-      <c r="B2" s="327" t="s">
+      <c r="B2" s="302" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="328"/>
-      <c r="D2" s="315" t="s">
+      <c r="C2" s="303"/>
+      <c r="D2" s="308" t="s">
         <v>335</v>
       </c>
-      <c r="E2" s="316"/>
-      <c r="F2" s="316"/>
-      <c r="G2" s="316"/>
-      <c r="H2" s="317"/>
+      <c r="E2" s="309"/>
+      <c r="F2" s="309"/>
+      <c r="G2" s="309"/>
+      <c r="H2" s="310"/>
     </row>
     <row r="3" spans="2:15">
-      <c r="B3" s="302" t="s">
+      <c r="B3" s="304" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="303"/>
-      <c r="D3" s="318" t="s">
+      <c r="C3" s="305"/>
+      <c r="D3" s="311" t="s">
         <v>322</v>
       </c>
-      <c r="E3" s="319"/>
-      <c r="F3" s="319"/>
-      <c r="G3" s="319"/>
-      <c r="H3" s="320"/>
-    </row>
-    <row r="4" spans="2:15" ht="13.8" thickBot="1">
-      <c r="B4" s="313" t="s">
+      <c r="E3" s="312"/>
+      <c r="F3" s="312"/>
+      <c r="G3" s="312"/>
+      <c r="H3" s="313"/>
+    </row>
+    <row r="4" spans="2:15" ht="14.25" thickBot="1">
+      <c r="B4" s="306" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="314"/>
-      <c r="D4" s="321" t="str">
+      <c r="C4" s="307"/>
+      <c r="D4" s="314" t="str">
         <f ca="1">表紙!D3&amp;".c"</f>
         <v>alert_S_ADBZR_ACC-CSTD-0-06-A-C0.c</v>
       </c>
-      <c r="E4" s="322"/>
-      <c r="F4" s="322"/>
-      <c r="G4" s="322"/>
-      <c r="H4" s="323"/>
-    </row>
-    <row r="5" spans="2:15" ht="13.8" thickBot="1">
+      <c r="E4" s="315"/>
+      <c r="F4" s="315"/>
+      <c r="G4" s="315"/>
+      <c r="H4" s="316"/>
+    </row>
+    <row r="5" spans="2:15" ht="14.25" thickBot="1">
       <c r="D5" t="str">
         <f ca="1">IF(LEN(表紙!D3&amp;".c") = LENB(表紙!D3&amp;".c"),"※モジュール名 全角チェックOK","※モジュール名 全角チェックNG：ファイル名に全角文字が使用されています！")</f>
         <v>※モジュール名 全角チェックOK</v>
       </c>
     </row>
     <row r="6" spans="2:15">
-      <c r="B6" s="327" t="s">
+      <c r="B6" s="302" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="328"/>
-      <c r="D6" s="324" t="str">
+      <c r="C6" s="303"/>
+      <c r="D6" s="317" t="str">
         <f ca="1">MID(D4, LEN("alert_") + 1, FIND("-",D4,1) - LEN("alert_") - 1)</f>
         <v>S_ADBZR_ACC</v>
       </c>
-      <c r="E6" s="325"/>
-      <c r="F6" s="325"/>
-      <c r="G6" s="325"/>
-      <c r="H6" s="326"/>
+      <c r="E6" s="318"/>
+      <c r="F6" s="318"/>
+      <c r="G6" s="318"/>
+      <c r="H6" s="319"/>
     </row>
     <row r="7" spans="2:15">
-      <c r="B7" s="302" t="s">
+      <c r="B7" s="304" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="303"/>
-      <c r="D7" s="304">
+      <c r="C7" s="305"/>
+      <c r="D7" s="320">
         <f>COUNTA($D$13:$D$37)</f>
         <v>1</v>
       </c>
-      <c r="E7" s="305"/>
-      <c r="F7" s="305"/>
-      <c r="G7" s="305"/>
-      <c r="H7" s="306"/>
-    </row>
-    <row r="8" spans="2:15" ht="14.4">
-      <c r="B8" s="302" t="s">
+      <c r="E7" s="321"/>
+      <c r="F7" s="321"/>
+      <c r="G7" s="321"/>
+      <c r="H7" s="322"/>
+    </row>
+    <row r="8" spans="2:15" ht="15">
+      <c r="B8" s="304" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="303"/>
-      <c r="D8" s="304" t="str">
+      <c r="C8" s="305"/>
+      <c r="D8" s="320" t="str">
         <f ca="1">"st_gp_ALERT_"&amp;UPPER(D6)&amp;"_MTRX"</f>
         <v>st_gp_ALERT_S_ADBZR_ACC_MTRX</v>
       </c>
-      <c r="E8" s="305"/>
-      <c r="F8" s="305"/>
-      <c r="G8" s="305"/>
-      <c r="H8" s="306"/>
+      <c r="E8" s="321"/>
+      <c r="F8" s="321"/>
+      <c r="G8" s="321"/>
+      <c r="H8" s="322"/>
       <c r="O8" s="279"/>
     </row>
     <row r="9" spans="2:15">
-      <c r="B9" s="302" t="s">
+      <c r="B9" s="304" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="303"/>
-      <c r="D9" s="307" t="s">
+      <c r="C9" s="305"/>
+      <c r="D9" s="323" t="s">
         <v>210</v>
       </c>
-      <c r="E9" s="308"/>
-      <c r="F9" s="308"/>
-      <c r="G9" s="308"/>
-      <c r="H9" s="309"/>
-    </row>
-    <row r="10" spans="2:15" ht="13.8" thickBot="1">
-      <c r="B10" s="313" t="s">
+      <c r="E9" s="324"/>
+      <c r="F9" s="324"/>
+      <c r="G9" s="324"/>
+      <c r="H9" s="325"/>
+    </row>
+    <row r="10" spans="2:15" ht="14.25" thickBot="1">
+      <c r="B10" s="306" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="314"/>
-      <c r="D10" s="310"/>
-      <c r="E10" s="311"/>
-      <c r="F10" s="311"/>
-      <c r="G10" s="311"/>
-      <c r="H10" s="312"/>
-    </row>
-    <row r="11" spans="2:15" ht="13.8" thickBot="1"/>
-    <row r="12" spans="2:15" ht="13.8" thickBot="1">
+      <c r="C10" s="307"/>
+      <c r="D10" s="326"/>
+      <c r="E10" s="327"/>
+      <c r="F10" s="327"/>
+      <c r="G10" s="327"/>
+      <c r="H10" s="328"/>
+    </row>
+    <row r="11" spans="2:15" ht="14.25" thickBot="1"/>
+    <row r="12" spans="2:15" ht="14.25" thickBot="1">
       <c r="B12" s="129" t="s">
         <v>34</v>
       </c>
@@ -11371,7 +11294,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="15" thickTop="1">
+    <row r="13" spans="2:15" ht="15.75" thickTop="1">
       <c r="B13" s="97">
         <v>1</v>
       </c>
@@ -12225,7 +12148,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:14" ht="13.8" thickBot="1">
+    <row r="37" spans="2:14" ht="14.25" thickBot="1">
       <c r="B37" s="88">
         <v>25</v>
       </c>
@@ -12265,22 +12188,22 @@
     <protectedRange sqref="D2:H3 D9:H10 C13:E37" name="編集許可"/>
   </protectedRanges>
   <mergeCells count="16">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <conditionalFormatting sqref="C13:C37">
@@ -12320,21 +12243,21 @@
     <tabColor rgb="FFCCFFCC"/>
   </sheetPr>
   <dimension ref="B2:R59"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="3.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="36.44140625" customWidth="1"/>
-    <col min="6" max="6" width="52.77734375" customWidth="1"/>
-    <col min="7" max="7" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="15" width="3.88671875" customWidth="1"/>
-    <col min="16" max="16" width="9.88671875" customWidth="1"/>
-    <col min="17" max="17" width="44.6640625" customWidth="1"/>
-    <col min="18" max="18" width="73.6640625" customWidth="1"/>
+    <col min="5" max="5" width="36.5" customWidth="1"/>
+    <col min="6" max="6" width="52.75" customWidth="1"/>
+    <col min="7" max="7" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="15" width="3.875" customWidth="1"/>
+    <col min="16" max="16" width="9.875" customWidth="1"/>
+    <col min="17" max="17" width="44.625" customWidth="1"/>
+    <col min="18" max="18" width="73.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" ht="13.8" thickBot="1">
+    <row r="2" spans="2:18" ht="14.25" thickBot="1">
       <c r="B2" t="s">
         <v>184</v>
       </c>
@@ -12342,7 +12265,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="3" spans="2:18" ht="13.8" thickBot="1">
+    <row r="3" spans="2:18" ht="14.25" thickBot="1">
       <c r="B3" s="129" t="s">
         <v>34</v>
       </c>
@@ -12380,7 +12303,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="4" spans="2:18" ht="13.8" hidden="1" thickTop="1">
+    <row r="4" spans="2:18" ht="14.25" hidden="1" thickTop="1">
       <c r="B4" s="158">
         <v>0</v>
       </c>
@@ -12408,7 +12331,7 @@
       </c>
       <c r="R4" s="128"/>
     </row>
-    <row r="5" spans="2:18" ht="13.8" thickTop="1">
+    <row r="5" spans="2:18" ht="14.25" thickTop="1">
       <c r="B5" s="161">
         <v>1</v>
       </c>
@@ -12936,7 +12859,7 @@
       <c r="Q28" s="133"/>
       <c r="R28" s="107"/>
     </row>
-    <row r="29" spans="2:18" ht="13.8" thickBot="1">
+    <row r="29" spans="2:18" ht="14.25" thickBot="1">
       <c r="B29" s="162">
         <v>25</v>
       </c>
@@ -12958,7 +12881,7 @@
       <c r="Q29" s="131"/>
       <c r="R29" s="109"/>
     </row>
-    <row r="32" spans="2:18" ht="13.8" thickBot="1">
+    <row r="32" spans="2:18" ht="14.25" thickBot="1">
       <c r="B32" t="s">
         <v>185</v>
       </c>
@@ -12966,7 +12889,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="33" spans="2:18" ht="13.8" thickBot="1">
+    <row r="33" spans="2:18" ht="14.25" thickBot="1">
       <c r="B33" s="129" t="s">
         <v>34</v>
       </c>
@@ -12998,7 +12921,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="2:18" ht="13.8" hidden="1" thickTop="1">
+    <row r="34" spans="2:18" ht="14.25" hidden="1" thickTop="1">
       <c r="B34" s="158">
         <v>0</v>
       </c>
@@ -13024,7 +12947,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="2:18" ht="13.8" thickTop="1">
+    <row r="35" spans="2:18" ht="14.25" thickTop="1">
       <c r="B35" s="161">
         <v>1</v>
       </c>
@@ -13552,7 +13475,7 @@
       <c r="Q58" s="133"/>
       <c r="R58" s="163"/>
     </row>
-    <row r="59" spans="2:18" ht="13.8" thickBot="1">
+    <row r="59" spans="2:18" ht="14.25" thickBot="1">
       <c r="B59" s="162">
         <v>25</v>
       </c>
@@ -13600,29 +13523,29 @@
     <tabColor rgb="FFCCFFCC"/>
   </sheetPr>
   <dimension ref="A1:U103"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" customWidth="1"/>
-    <col min="6" max="6" width="19.77734375" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" customWidth="1"/>
-    <col min="8" max="8" width="30.44140625" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" customWidth="1"/>
-    <col min="10" max="10" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" customWidth="1"/>
-    <col min="12" max="12" width="16.109375" customWidth="1"/>
-    <col min="14" max="14" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.109375" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="28.375" customWidth="1"/>
+    <col min="3" max="3" width="15.875" customWidth="1"/>
+    <col min="5" max="5" width="12.375" customWidth="1"/>
+    <col min="6" max="6" width="19.75" customWidth="1"/>
+    <col min="7" max="7" width="12.375" customWidth="1"/>
+    <col min="8" max="8" width="30.5" customWidth="1"/>
+    <col min="9" max="9" width="12.375" customWidth="1"/>
+    <col min="10" max="10" width="32.25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.375" customWidth="1"/>
+    <col min="12" max="12" width="16.125" customWidth="1"/>
+    <col min="14" max="14" width="30.125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="57.125" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="13.8" thickBot="1">
+    <row r="1" spans="1:21" ht="14.25" thickBot="1">
       <c r="C1" s="81" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="13.8" thickBot="1">
+    <row r="2" spans="1:21" ht="14.25" thickBot="1">
       <c r="B2" s="89" t="s">
         <v>58</v>
       </c>
@@ -13666,7 +13589,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="14.4" hidden="1" thickTop="1" thickBot="1">
+    <row r="3" spans="1:21" ht="15" hidden="1" thickTop="1" thickBot="1">
       <c r="B3" s="24"/>
       <c r="C3" s="43" t="s">
         <v>107</v>
@@ -13687,7 +13610,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="13.8" thickTop="1">
+    <row r="4" spans="1:21" ht="14.25" thickTop="1">
       <c r="A4" s="81" t="s">
         <v>336</v>
       </c>
@@ -14108,7 +14031,7 @@
       </c>
       <c r="U12" s="28"/>
     </row>
-    <row r="13" spans="1:21" ht="13.8" thickBot="1">
+    <row r="13" spans="1:21" ht="14.25" thickBot="1">
       <c r="B13" s="24"/>
       <c r="C13" s="23"/>
       <c r="D13" s="106"/>
@@ -16359,7 +16282,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="103" spans="2:15" ht="13.8" thickBot="1">
+    <row r="103" spans="2:15" ht="14.25" thickBot="1">
       <c r="B103" s="45"/>
       <c r="C103" s="46"/>
       <c r="D103" s="108"/>
@@ -16428,18 +16351,18 @@
     <tabColor rgb="FFCCECFF"/>
   </sheetPr>
   <dimension ref="A1:AW199"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="3" bestFit="1" customWidth="1"/>
     <col min="4" max="35" width="3" customWidth="1"/>
-    <col min="36" max="36" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="4.109375" customWidth="1"/>
+    <col min="36" max="36" width="36.375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="4.125" customWidth="1"/>
     <col min="38" max="42" width="9" hidden="1" customWidth="1"/>
-    <col min="43" max="43" width="20.6640625" hidden="1" customWidth="1"/>
-    <col min="44" max="47" width="41.109375" customWidth="1"/>
-    <col min="48" max="48" width="23.6640625" customWidth="1"/>
+    <col min="43" max="43" width="20.625" hidden="1" customWidth="1"/>
+    <col min="44" max="47" width="41.125" customWidth="1"/>
+    <col min="48" max="48" width="23.625" customWidth="1"/>
     <col min="49" max="49" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16657,7 +16580,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:49" ht="13.8" thickBot="1">
+    <row r="4" spans="1:49" ht="14.25" thickBot="1">
       <c r="A4" s="333" t="s">
         <v>63</v>
       </c>
@@ -16705,7 +16628,7 @@
       <c r="AV4" s="71"/>
       <c r="AW4" s="72"/>
     </row>
-    <row r="5" spans="1:49" ht="13.8" thickBot="1">
+    <row r="5" spans="1:49" ht="14.25" thickBot="1">
       <c r="A5" s="335"/>
       <c r="B5" s="336"/>
       <c r="C5" s="199"/>
@@ -18225,7 +18148,7 @@
         <v>ALERT_VOM_IGN_ON</v>
       </c>
     </row>
-    <row r="17" spans="2:49" ht="13.8" thickBot="1">
+    <row r="17" spans="2:49" ht="14.25" thickBot="1">
       <c r="B17" s="124"/>
       <c r="C17" s="39">
         <f t="shared" si="2"/>
@@ -24701,7 +24624,7 @@
         <v xml:space="preserve">    (U1)ALERT_REQ_UNKNOWN                                                      /* 63 UNKNOWN                                         */</v>
       </c>
     </row>
-    <row r="70" spans="1:46" ht="13.8" thickBot="1">
+    <row r="70" spans="1:46" ht="14.25" thickBot="1">
       <c r="A70" s="48" t="s">
         <v>64</v>
       </c>
@@ -45327,19 +45250,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A11:CD366"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="139.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="10" width="3.33203125" customWidth="1"/>
-    <col min="11" max="11" width="21.33203125" customWidth="1"/>
-    <col min="12" max="12" width="45.109375" customWidth="1"/>
+    <col min="2" max="2" width="139.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="10" width="3.375" customWidth="1"/>
+    <col min="11" max="11" width="21.375" customWidth="1"/>
+    <col min="12" max="12" width="45.125" customWidth="1"/>
     <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="14" width="78.109375" customWidth="1"/>
-    <col min="15" max="15" width="24.77734375" customWidth="1"/>
-    <col min="16" max="16" width="37.88671875" customWidth="1"/>
-    <col min="17" max="17" width="30.6640625" customWidth="1"/>
-    <col min="18" max="18" width="10.88671875" customWidth="1"/>
-    <col min="19" max="19" width="14.33203125" customWidth="1"/>
+    <col min="14" max="14" width="78.125" customWidth="1"/>
+    <col min="15" max="15" width="24.75" customWidth="1"/>
+    <col min="16" max="16" width="37.875" customWidth="1"/>
+    <col min="17" max="17" width="30.625" customWidth="1"/>
+    <col min="18" max="18" width="10.875" customWidth="1"/>
+    <col min="19" max="19" width="14.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="11" spans="2:17">
@@ -45936,7 +45859,7 @@
       <c r="P43" s="38"/>
       <c r="Q43" s="38"/>
     </row>
-    <row r="44" spans="2:82" ht="14.4">
+    <row r="44" spans="2:82" ht="14.25">
       <c r="B44" s="38"/>
       <c r="C44" s="38"/>
       <c r="D44" s="38"/>
@@ -46667,7 +46590,7 @@
       <c r="Q75" s="212"/>
       <c r="R75" s="52"/>
     </row>
-    <row r="76" spans="1:21" ht="26.4">
+    <row r="76" spans="1:21" ht="27">
       <c r="B76" s="64" t="s">
         <v>27</v>
       </c>
@@ -46694,7 +46617,7 @@
       <c r="Q76" s="217"/>
       <c r="R76" s="52"/>
     </row>
-    <row r="77" spans="1:21" ht="133.19999999999999">
+    <row r="77" spans="1:21" ht="136.5">
       <c r="B77" s="63" t="s">
         <v>28</v>
       </c>
@@ -46785,7 +46708,7 @@
       <c r="Q78" s="220"/>
       <c r="R78" s="52"/>
     </row>
-    <row r="79" spans="1:21" ht="13.8" thickTop="1">
+    <row r="79" spans="1:21" ht="14.25" thickTop="1">
       <c r="B79" s="66" t="s">
         <v>232</v>
       </c>
@@ -47313,7 +47236,7 @@
       </c>
       <c r="Q90" s="221"/>
     </row>
-    <row r="91" spans="2:17" ht="13.8" thickBot="1">
+    <row r="91" spans="2:17" ht="14.25" thickBot="1">
       <c r="B91" s="189" t="s">
         <v>243</v>
       </c>
@@ -47379,59 +47302,59 @@
       <c r="Q98" s="218"/>
     </row>
     <row r="107" spans="17:17" ht="13.5" customHeight="1"/>
-    <row r="109" spans="17:17" ht="12.9" customHeight="1"/>
-    <row r="111" spans="17:17" ht="12.9" customHeight="1"/>
-    <row r="112" spans="17:17" ht="12.9" customHeight="1"/>
-    <row r="113" ht="12.9" customHeight="1"/>
-    <row r="114" ht="12.9" customHeight="1"/>
-    <row r="115" ht="12.9" customHeight="1"/>
-    <row r="116" ht="12.9" customHeight="1"/>
-    <row r="117" ht="12.9" customHeight="1"/>
-    <row r="118" ht="12.9" customHeight="1"/>
-    <row r="119" ht="12.9" customHeight="1"/>
-    <row r="120" ht="12.9" customHeight="1"/>
-    <row r="121" ht="12.9" customHeight="1"/>
-    <row r="122" ht="12.9" customHeight="1"/>
-    <row r="123" ht="12.9" customHeight="1"/>
-    <row r="125" ht="12.9" customHeight="1"/>
-    <row r="126" ht="12.9" customHeight="1"/>
-    <row r="127" ht="12.9" customHeight="1"/>
-    <row r="128" ht="12.9" customHeight="1"/>
-    <row r="129" ht="12.9" customHeight="1"/>
-    <row r="130" ht="12.9" customHeight="1"/>
-    <row r="131" ht="12.9" customHeight="1"/>
-    <row r="132" ht="12.9" customHeight="1"/>
-    <row r="133" ht="12.9" customHeight="1"/>
-    <row r="134" ht="12.9" customHeight="1"/>
-    <row r="135" ht="12.9" customHeight="1"/>
-    <row r="136" ht="12.9" customHeight="1"/>
-    <row r="137" ht="12.9" customHeight="1"/>
-    <row r="138" ht="12.9" customHeight="1"/>
-    <row r="140" ht="12.9" customHeight="1"/>
-    <row r="141" ht="12.9" customHeight="1"/>
-    <row r="142" ht="12.9" customHeight="1"/>
-    <row r="143" ht="12.9" customHeight="1"/>
-    <row r="144" ht="12.9" customHeight="1"/>
-    <row r="145" ht="12.9" customHeight="1"/>
-    <row r="146" ht="12.9" customHeight="1"/>
-    <row r="147" ht="12.9" customHeight="1"/>
-    <row r="148" ht="12.9" customHeight="1"/>
-    <row r="149" ht="12.9" customHeight="1"/>
-    <row r="150" ht="12.9" customHeight="1"/>
-    <row r="151" ht="12.9" customHeight="1"/>
-    <row r="152" ht="12.9" customHeight="1"/>
-    <row r="153" ht="12.9" customHeight="1"/>
-    <row r="155" ht="12.9" customHeight="1"/>
-    <row r="156" ht="12.9" customHeight="1"/>
-    <row r="157" ht="12.9" customHeight="1"/>
-    <row r="158" ht="12.9" customHeight="1"/>
-    <row r="159" ht="12.9" customHeight="1"/>
-    <row r="160" ht="12.9" customHeight="1"/>
-    <row r="161" ht="12.9" customHeight="1"/>
-    <row r="162" ht="12.9" customHeight="1"/>
-    <row r="163" ht="12.9" customHeight="1"/>
-    <row r="164" ht="12.9" customHeight="1"/>
-    <row r="165" ht="12.9" customHeight="1"/>
+    <row r="109" spans="17:17" ht="12.95" customHeight="1"/>
+    <row r="111" spans="17:17" ht="12.95" customHeight="1"/>
+    <row r="112" spans="17:17" ht="12.95" customHeight="1"/>
+    <row r="113" ht="12.95" customHeight="1"/>
+    <row r="114" ht="12.95" customHeight="1"/>
+    <row r="115" ht="12.95" customHeight="1"/>
+    <row r="116" ht="12.95" customHeight="1"/>
+    <row r="117" ht="12.95" customHeight="1"/>
+    <row r="118" ht="12.95" customHeight="1"/>
+    <row r="119" ht="12.95" customHeight="1"/>
+    <row r="120" ht="12.95" customHeight="1"/>
+    <row r="121" ht="12.95" customHeight="1"/>
+    <row r="122" ht="12.95" customHeight="1"/>
+    <row r="123" ht="12.95" customHeight="1"/>
+    <row r="125" ht="12.95" customHeight="1"/>
+    <row r="126" ht="12.95" customHeight="1"/>
+    <row r="127" ht="12.95" customHeight="1"/>
+    <row r="128" ht="12.95" customHeight="1"/>
+    <row r="129" ht="12.95" customHeight="1"/>
+    <row r="130" ht="12.95" customHeight="1"/>
+    <row r="131" ht="12.95" customHeight="1"/>
+    <row r="132" ht="12.95" customHeight="1"/>
+    <row r="133" ht="12.95" customHeight="1"/>
+    <row r="134" ht="12.95" customHeight="1"/>
+    <row r="135" ht="12.95" customHeight="1"/>
+    <row r="136" ht="12.95" customHeight="1"/>
+    <row r="137" ht="12.95" customHeight="1"/>
+    <row r="138" ht="12.95" customHeight="1"/>
+    <row r="140" ht="12.95" customHeight="1"/>
+    <row r="141" ht="12.95" customHeight="1"/>
+    <row r="142" ht="12.95" customHeight="1"/>
+    <row r="143" ht="12.95" customHeight="1"/>
+    <row r="144" ht="12.95" customHeight="1"/>
+    <row r="145" ht="12.95" customHeight="1"/>
+    <row r="146" ht="12.95" customHeight="1"/>
+    <row r="147" ht="12.95" customHeight="1"/>
+    <row r="148" ht="12.95" customHeight="1"/>
+    <row r="149" ht="12.95" customHeight="1"/>
+    <row r="150" ht="12.95" customHeight="1"/>
+    <row r="151" ht="12.95" customHeight="1"/>
+    <row r="152" ht="12.95" customHeight="1"/>
+    <row r="153" ht="12.95" customHeight="1"/>
+    <row r="155" ht="12.95" customHeight="1"/>
+    <row r="156" ht="12.95" customHeight="1"/>
+    <row r="157" ht="12.95" customHeight="1"/>
+    <row r="158" ht="12.95" customHeight="1"/>
+    <row r="159" ht="12.95" customHeight="1"/>
+    <row r="160" ht="12.95" customHeight="1"/>
+    <row r="161" ht="12.95" customHeight="1"/>
+    <row r="162" ht="12.95" customHeight="1"/>
+    <row r="163" ht="12.95" customHeight="1"/>
+    <row r="164" ht="12.95" customHeight="1"/>
+    <row r="165" ht="12.95" customHeight="1"/>
     <row r="366" ht="144" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
@@ -47455,14 +47378,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="B2:D27"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" customWidth="1"/>
+    <col min="2" max="2" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.25" customWidth="1"/>
     <col min="4" max="4" width="86" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="13.8" thickBot="1">
+    <row r="2" spans="2:4" ht="14.25" thickBot="1">
       <c r="B2" s="74" t="s">
         <v>84</v>
       </c>
@@ -47472,7 +47395,7 @@
       </c>
       <c r="D2" s="75"/>
     </row>
-    <row r="3" spans="2:4" ht="13.8" thickBot="1">
+    <row r="3" spans="2:4" ht="14.25" thickBot="1">
       <c r="B3" s="68" t="s">
         <v>84</v>
       </c>
@@ -47483,7 +47406,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="13.8" thickTop="1">
+    <row r="4" spans="2:4" ht="14.25" thickTop="1">
       <c r="B4" s="12">
         <v>0</v>
       </c>
@@ -47494,7 +47417,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="39.6">
+    <row r="5" spans="2:4" ht="40.5">
       <c r="B5" s="2">
         <v>1</v>
       </c>
@@ -47505,7 +47428,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="26.4">
+    <row r="6" spans="2:4" ht="27">
       <c r="B6" s="2">
         <v>2</v>
       </c>
@@ -47516,7 +47439,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="52.8">
+    <row r="7" spans="2:4" ht="54">
       <c r="B7" s="2">
         <v>3</v>
       </c>
@@ -47527,7 +47450,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="79.2">
+    <row r="8" spans="2:4" ht="81">
       <c r="B8" s="2">
         <v>4</v>
       </c>
@@ -47549,7 +47472,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="26.4">
+    <row r="10" spans="2:4" ht="27">
       <c r="B10" s="2">
         <v>6</v>
       </c>
@@ -47560,7 +47483,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="26.4">
+    <row r="11" spans="2:4" ht="27">
       <c r="B11" s="2">
         <v>7</v>
       </c>
@@ -47571,7 +47494,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="26.4">
+    <row r="12" spans="2:4" ht="27">
       <c r="B12" s="2">
         <v>8</v>
       </c>
@@ -47582,7 +47505,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="26.4">
+    <row r="13" spans="2:4" ht="27">
       <c r="B13" s="2">
         <v>9</v>
       </c>
@@ -47593,7 +47516,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="26.4">
+    <row r="14" spans="2:4" ht="27">
       <c r="B14" s="2">
         <v>10</v>
       </c>
@@ -47604,7 +47527,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="132">
+    <row r="15" spans="2:4" ht="135">
       <c r="B15" s="2">
         <v>11</v>
       </c>
@@ -47626,7 +47549,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="26.4">
+    <row r="17" spans="2:4" ht="27">
       <c r="B17" s="2">
         <v>13</v>
       </c>
@@ -47637,7 +47560,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="92.4">
+    <row r="18" spans="2:4" ht="67.5">
       <c r="B18" s="2">
         <v>14</v>
       </c>
@@ -47648,7 +47571,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="39.6">
+    <row r="19" spans="2:4" ht="40.5">
       <c r="B19" s="2">
         <v>15</v>
       </c>
@@ -47681,7 +47604,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="26.4">
+    <row r="22" spans="2:4" ht="27">
       <c r="B22" s="2">
         <v>18</v>
       </c>
@@ -47692,7 +47615,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23" spans="2:4" ht="26.4">
+    <row r="23" spans="2:4" ht="27">
       <c r="B23" s="2">
         <v>19</v>
       </c>
@@ -47703,7 +47626,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="24" spans="2:4" ht="92.4">
+    <row r="24" spans="2:4" ht="94.5">
       <c r="B24" s="214">
         <v>20</v>
       </c>
@@ -47724,7 +47647,7 @@
       <c r="C26" s="78"/>
       <c r="D26" s="67"/>
     </row>
-    <row r="27" spans="2:4" ht="13.8" thickBot="1">
+    <row r="27" spans="2:4" ht="14.25" thickBot="1">
       <c r="B27" s="4"/>
       <c r="C27" s="79"/>
       <c r="D27" s="5"/>

</xml_diff>